<commit_message>
feat: Add end-to-end tests for dashboard, manage account, new ticket, organization settings, and ticket detail pages
- Implement DashboardPage class for dashboard interactions and assertions
- Create ManageAccountPage class for managing user details and security settings
- Develop NewTicketPage class for submitting new tickets and validating form inputs
- Introduce OrganizationSettingsPage class for managing organization members
- Add TicketDetailPage class for viewing ticket details and status updates
- Write comprehensive test suites for dashboard layout, navigation, search & filter functionality
- Create tests for managing account details and security settings
- Implement tests for new ticket form rendering and validation
- Add tests for organization settings member management
- Develop tests for ticket detail dialog interactions and assertions
</commit_message>
<xml_diff>
--- a/manual/TEST-CASES.xlsx
+++ b/manual/TEST-CASES.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="432">
   <si>
     <t>Test ID</t>
   </si>
@@ -99,7 +99,7 @@
     <t>Happy Path</t>
   </si>
   <si>
-    <t>2026-05-24</t>
+    <t>2026-05-25</t>
   </si>
   <si>
     <t>AutoQA</t>
@@ -327,6 +327,834 @@
 3. Assert URL still /sign-in.</t>
   </si>
   <si>
+    <t>DB0001</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>User lands on /&lt;slug&gt;/tickets with all core chrome visible</t>
+  </si>
+  <si>
+    <t>Post-login default landing — tickets list page must render search, filter, New button, and header avatar.</t>
+  </si>
+  <si>
+    <t>Signed in with at least one organization (storage state from globalSetup).</t>
+  </si>
+  <si>
+    <t>org slug captured during globalSetup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to /&lt;slug&gt;/tickets.
+2. Assert search, status filter, New link, user-menu trigger, org switcher all visible.
+3. Assert URL ends with /&lt;slug&gt;/tickets.</t>
+  </si>
+  <si>
+    <t>All five chrome elements visible; URL matches.</t>
+  </si>
+  <si>
+    <t>e2e/tests/dashboard.spec.ts</t>
+  </si>
+  <si>
+    <t>DB0002</t>
+  </si>
+  <si>
+    <t>Header has Tickets and Settings tabs, Tickets is active by default</t>
+  </si>
+  <si>
+    <t>Confirms tab routing structure and default selection.</t>
+  </si>
+  <si>
+    <t>On /&lt;slug&gt;/tickets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Assert both header tabs visible.
+2. Assert aria-selected=true on Tickets tab.</t>
+  </si>
+  <si>
+    <t>Two tabs present; Tickets selected.</t>
+  </si>
+  <si>
+    <t>UI and validation</t>
+  </si>
+  <si>
+    <t>DB0003</t>
+  </si>
+  <si>
+    <t>Sidebar nav exposes Tickets, Organization settings, Manage account, Sign out</t>
+  </si>
+  <si>
+    <t>Sidebar NavLinks must always be visible while signed in.</t>
+  </si>
+  <si>
+    <t>1. Assert each of the four NavLinks visible by text inside &lt;nav&gt;.</t>
+  </si>
+  <si>
+    <t>All four NavLinks present.</t>
+  </si>
+  <si>
+    <t>DB0004</t>
+  </si>
+  <si>
+    <t>Seeded sample tickets are findable in the org's ticket list</t>
+  </si>
+  <si>
+    <t>After "Import example tickets", the seed row "Session timeout not working correctly" must be findable via search regardless of how many newer tickets E2E runs have added.</t>
+  </si>
+  <si>
+    <t>Org was bootstrapped with the sample-tickets import.</t>
+  </si>
+  <si>
+    <t>Seed title: "Session timeout not working correctly".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search the table for the seeded title.
+2. Assert the row is rendered.</t>
+  </si>
+  <si>
+    <t>Seeded row visible after search.</t>
+  </si>
+  <si>
+    <t>DB0005</t>
+  </si>
+  <si>
+    <t>Clicking "Settings" header tab routes to /&lt;slug&gt;/settings</t>
+  </si>
+  <si>
+    <t>Header tab routing works for Settings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Settings tab.
+2. Wait for URL change.</t>
+  </si>
+  <si>
+    <t>URL ends /&lt;slug&gt;/settings.</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>DB0006</t>
+  </si>
+  <si>
+    <t>Clicking "New" routes to /&lt;slug&gt;/tickets/new</t>
+  </si>
+  <si>
+    <t>Authenticated user can navigate to the new-ticket form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click "New" link.
+2. Wait for URL change.</t>
+  </si>
+  <si>
+    <t>URL ends /&lt;slug&gt;/tickets/new.</t>
+  </si>
+  <si>
+    <t>DB0007</t>
+  </si>
+  <si>
+    <t>Search by title puts the term in ?search and narrows the table</t>
+  </si>
+  <si>
+    <t>Search input + Enter triggers a tRPC refetch with the new search param; URL gains ?search=...</t>
+  </si>
+  <si>
+    <t>Search term: "Session timeout" (matches exactly one seed row).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Type term in search input.
+2. Press Enter.
+3. Wait for tickets.getList response.
+4. Assert URL contains search param.
+5. Assert exactly 1 row visible.</t>
+  </si>
+  <si>
+    <t>?search=Session+timeout in URL; 1 row in table.</t>
+  </si>
+  <si>
+    <t>DB0008</t>
+  </si>
+  <si>
+    <t>Search with a guaranteed-unique gibberish term yields zero rows</t>
+  </si>
+  <si>
+    <t>Empty-results state — search that matches nothing must render no ticket rows.</t>
+  </si>
+  <si>
+    <t>Search term: "zzzz_no_such_ticket_9921".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search gibberish term.
+2. Assert URL contains search param.
+3. Assert 0 rows.</t>
+  </si>
+  <si>
+    <t>0 rows.</t>
+  </si>
+  <si>
+    <t>DB0009</t>
+  </si>
+  <si>
+    <t>Status filter "In Progress" sets ?status=InProgress and shows only matching rows</t>
+  </si>
+  <si>
+    <t>Status filter narrows the table to rows matching the chosen status.</t>
+  </si>
+  <si>
+    <t>Filter value: "In Progress".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open status filter.
+2. Pick "In Progress".
+3. Assert URL contains ?status=InProgress.
+4. Assert every visible status badge reads "In Progress".</t>
+  </si>
+  <si>
+    <t>?status=InProgress; all badges match.</t>
+  </si>
+  <si>
+    <t>Filtering</t>
+  </si>
+  <si>
+    <t>DB0010</t>
+  </si>
+  <si>
+    <t>Reverting the status filter to "Any" clears ?status from the URL</t>
+  </si>
+  <si>
+    <t>Picking "Any" must remove the status URL param entirely.</t>
+  </si>
+  <si>
+    <t>On /&lt;slug&gt;/tickets with status filter active.</t>
+  </si>
+  <si>
+    <t>Filter value: "Any".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Pick "In Progress".
+2. Pick "Any".
+3. Assert URL has no ?status param.</t>
+  </si>
+  <si>
+    <t>No ?status= in URL.</t>
+  </si>
+  <si>
+    <t>TK0001</t>
+  </si>
+  <si>
+    <t>Ticket Detail</t>
+  </si>
+  <si>
+    <t>Clicking a ticket row opens the detail dialog with all core fields</t>
+  </si>
+  <si>
+    <t>The dialog must render title, status combobox, description, ID, reporter, created date, and Comments section.</t>
+  </si>
+  <si>
+    <t>On /&lt;slug&gt;/tickets with the seed row searchable.</t>
+  </si>
+  <si>
+    <t>Seed title "Session timeout not working correctly".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search for the seed title.
+2. Click the row.
+3. Assert dialog open.
+4. Assert title + every core field visible.</t>
+  </si>
+  <si>
+    <t>Dialog renders all six core fields.</t>
+  </si>
+  <si>
+    <t>e2e/tests/ticketDetail.spec.ts</t>
+  </si>
+  <si>
+    <t>TK0002</t>
+  </si>
+  <si>
+    <t>URL gains ?selectedId=&lt;id&gt; while the dialog is open</t>
+  </si>
+  <si>
+    <t>The dialog open state is reflected in the URL via ?selectedId so the page is deep-linkable.</t>
+  </si>
+  <si>
+    <t>Dialog open via row click.</t>
+  </si>
+  <si>
+    <t>1. Assert ?selectedId in URL matches a ticket id ([a-z0-9]+).</t>
+  </si>
+  <si>
+    <t>selectedId search param present.</t>
+  </si>
+  <si>
+    <t>TK0003</t>
+  </si>
+  <si>
+    <t>Dialog status button shows the ticket's current status</t>
+  </si>
+  <si>
+    <t>Status combobox label reflects the ticket's current status from the API.</t>
+  </si>
+  <si>
+    <t>Dialog open for the seed ticket (status: In Progress).</t>
+  </si>
+  <si>
+    <t>Seed ticket status "In Progress".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Read status button text.
+2. Assert it contains "In Progress".</t>
+  </si>
+  <si>
+    <t>Status button shows "In Progress".</t>
+  </si>
+  <si>
+    <t>TK0004</t>
+  </si>
+  <si>
+    <t>Opening the status menu reveals all four status options</t>
+  </si>
+  <si>
+    <t>Status combobox must expose exactly New / In Progress / Resolved / Closed.</t>
+  </si>
+  <si>
+    <t>Dialog open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click status combobox.
+2. Assert all four options visible.
+3. Assert no extra options.</t>
+  </si>
+  <si>
+    <t>Exactly 4 .mantine-Combobox-option entries.</t>
+  </si>
+  <si>
+    <t>TK0005</t>
+  </si>
+  <si>
+    <t>Close (X) button closes the dialog and clears ?selectedId</t>
+  </si>
+  <si>
+    <t>Clicking the close ActionIcon removes the dialog and clears the URL param.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click close (X).
+2. Assert dialog detached.
+3. Assert ?selectedId is gone.</t>
+  </si>
+  <si>
+    <t>Dialog count 0; param removed.</t>
+  </si>
+  <si>
+    <t>TK0006</t>
+  </si>
+  <si>
+    <t>Empty ticket shows "No comments yet" placeholder and comment input</t>
+  </si>
+  <si>
+    <t>For tickets with zero comments, the dialog renders an empty-state and the Add-a-comment input + Send button.</t>
+  </si>
+  <si>
+    <t>Dialog open on a comment-free ticket.</t>
+  </si>
+  <si>
+    <t>Seed ticket has 0 comments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Assert "No comments yet" placeholder.
+2. Assert add-a-comment textbox visible.
+3. Assert Send button visible.</t>
+  </si>
+  <si>
+    <t>Empty-state + comment-entry UI present.</t>
+  </si>
+  <si>
+    <t>NT0001</t>
+  </si>
+  <si>
+    <t>New Ticket</t>
+  </si>
+  <si>
+    <t>The submit form renders all four required fields</t>
+  </si>
+  <si>
+    <t>Customer-facing public form must always expose reportedBy / yourName / title / description / Submit.</t>
+  </si>
+  <si>
+    <t>Navigate to /&lt;slug&gt;/tickets/new.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open page.
+2. Assert all four textboxes + Submit visible.</t>
+  </si>
+  <si>
+    <t>All five elements visible.</t>
+  </si>
+  <si>
+    <t>e2e/tests/newTicket.spec.ts</t>
+  </si>
+  <si>
+    <t>NT0002</t>
+  </si>
+  <si>
+    <t>Submitting an empty form shows validation errors on every field</t>
+  </si>
+  <si>
+    <t>Client-side validation blocks blank submissions on every required field.</t>
+  </si>
+  <si>
+    <t>On /&lt;slug&gt;/tickets/new.</t>
+  </si>
+  <si>
+    <t>None (empty form).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Submit.
+2. Assert "Invalid email" + ≥3 "String must contain at least 1 character(s)" errors.
+3. Assert URL unchanged.</t>
+  </si>
+  <si>
+    <t>All required-field errors visible; no API call.</t>
+  </si>
+  <si>
+    <t>NT0003</t>
+  </si>
+  <si>
+    <t>Submitting with a malformed reported-by email shows "Invalid email"</t>
+  </si>
+  <si>
+    <t>Email-format validation rejects malformed input before submit.</t>
+  </si>
+  <si>
+    <t>Email: "notanemail" + valid other fields.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fill all fields with malformed email.
+2. Submit.
+3. Assert "Invalid email" error.
+4. Assert URL unchanged.</t>
+  </si>
+  <si>
+    <t>Inline email error; no navigation.</t>
+  </si>
+  <si>
+    <t>NT0004</t>
+  </si>
+  <si>
+    <t>Valid submission shows the success toast and lands on the new ticket's detail page</t>
+  </si>
+  <si>
+    <t>Happy path: valid form creates a ticket and redirects to /&lt;slug&gt;/tickets/&lt;id&gt;.</t>
+  </si>
+  <si>
+    <t>Email "qa-bot@example.com", title "NT0004 e2e probe &lt;timestamp&gt;", body text.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fill all four fields.
+2. Submit.
+3. Assert toast.
+4. Assert URL matches /tickets/&lt;id&gt;.</t>
+  </si>
+  <si>
+    <t>Toast + detail-page URL.</t>
+  </si>
+  <si>
+    <t>Creates real ticket each run; non-destructive (no DELETE endpoint).</t>
+  </si>
+  <si>
+    <t>OS0001</t>
+  </si>
+  <si>
+    <t>Organization Settings</t>
+  </si>
+  <si>
+    <t>Page renders the "Organization members" heading and an "Add member" button</t>
+  </si>
+  <si>
+    <t>Settings page chrome: heading + primary CTA.</t>
+  </si>
+  <si>
+    <t>On /&lt;slug&gt;/settings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Assert "Organization members" heading.
+2. Assert "Add member" button.</t>
+  </si>
+  <si>
+    <t>Both visible.</t>
+  </si>
+  <si>
+    <t>e2e/tests/organizationSettings.spec.ts</t>
+  </si>
+  <si>
+    <t>OS0002</t>
+  </si>
+  <si>
+    <t>Logged-in user is listed as an Admin in the members roster</t>
+  </si>
+  <si>
+    <t>The org creator must appear in the members list with role=Admin.</t>
+  </si>
+  <si>
+    <t>Test account is the org creator.</t>
+  </si>
+  <si>
+    <t>Credentials.valid.email.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Assert the user's email appears in the roster.
+2. Assert "Admin" text appears in main.</t>
+  </si>
+  <si>
+    <t>Email + Admin label visible.</t>
+  </si>
+  <si>
+    <t>Authorization</t>
+  </si>
+  <si>
+    <t>OS0003</t>
+  </si>
+  <si>
+    <t>"Add member" opens a dialog with Email + Role inputs and submit button</t>
+  </si>
+  <si>
+    <t>Add-member modal renders all expected controls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click "Add member".
+2. Assert dialog open.
+3. Assert email input, role combobox, submit button visible.
+4. Close.</t>
+  </si>
+  <si>
+    <t>Dialog with three controls.</t>
+  </si>
+  <si>
+    <t>OS0004</t>
+  </si>
+  <si>
+    <t>Submitting the Add Member dialog with empty email shows "Invalid email"</t>
+  </si>
+  <si>
+    <t>Email required — empty submission blocked client-side.</t>
+  </si>
+  <si>
+    <t>Add-member dialog open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click submit with empty email.
+2. Assert "Invalid email" error inside dialog.
+3. Close.</t>
+  </si>
+  <si>
+    <t>Inline error; no invite sent.</t>
+  </si>
+  <si>
+    <t>OS0005</t>
+  </si>
+  <si>
+    <t>Submitting with a malformed email shows "Invalid email" without sending the invite</t>
+  </si>
+  <si>
+    <t>Email-format check rejects "notanemail" before submitting.</t>
+  </si>
+  <si>
+    <t>Email "notanemail".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fill malformed email.
+2. Submit.
+3. Assert "Invalid email" error.
+4. Assert dialog still open.</t>
+  </si>
+  <si>
+    <t>Dialog stays open; error visible.</t>
+  </si>
+  <si>
+    <t>OS0006</t>
+  </si>
+  <si>
+    <t>Role dropdown exposes both Admin and Member options</t>
+  </si>
+  <si>
+    <t>Add-member dialog allows choosing Admin or Member.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Role dropdown.
+2. Assert both options visible.
+3. Close.</t>
+  </si>
+  <si>
+    <t>Two role options.</t>
+  </si>
+  <si>
+    <t>OS0007</t>
+  </si>
+  <si>
+    <t>Closing the dialog removes it from the DOM</t>
+  </si>
+  <si>
+    <t>Dialog close button (X) detaches the modal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click close (X).
+2. Assert dialog count == 0.</t>
+  </si>
+  <si>
+    <t>No dialog in DOM.</t>
+  </si>
+  <si>
+    <t>MA0001</t>
+  </si>
+  <si>
+    <t>Manage Account</t>
+  </si>
+  <si>
+    <t>User details tab renders First name, Last name, Save</t>
+  </si>
+  <si>
+    <t>Profile edit form must always expose the name fields and save button.</t>
+  </si>
+  <si>
+    <t>On /manage-account.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open page.
+2. Assert First name, Last name, Save visible.</t>
+  </si>
+  <si>
+    <t>All three controls visible.</t>
+  </si>
+  <si>
+    <t>e2e/tests/manageAccount.spec.ts</t>
+  </si>
+  <si>
+    <t>MA0002</t>
+  </si>
+  <si>
+    <t>First name and Last name are pre-filled from the logged-in user's profile</t>
+  </si>
+  <si>
+    <t>Form pre-fills with session data so user can edit in place.</t>
+  </si>
+  <si>
+    <t>Signed in.</t>
+  </si>
+  <si>
+    <t>session.user.firstName / lastName.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Read inputValue() from First name and Last name fields.
+2. Assert both non-empty.</t>
+  </si>
+  <si>
+    <t>Both inputs have values.</t>
+  </si>
+  <si>
+    <t>MA0003</t>
+  </si>
+  <si>
+    <t>The page exposes both "User details" and "Security" tabs</t>
+  </si>
+  <si>
+    <t>Tab navigation between profile and password sections.</t>
+  </si>
+  <si>
+    <t>1. Assert both tabs visible.</t>
+  </si>
+  <si>
+    <t>Both tabs present.</t>
+  </si>
+  <si>
+    <t>MA0004</t>
+  </si>
+  <si>
+    <t>Security tab renders Sessions list section heading</t>
+  </si>
+  <si>
+    <t>Security tab must always show the Sessions section, even when the list is empty (no other devices).</t>
+  </si>
+  <si>
+    <t>On /manage-account, Security tab active.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Security tab.
+2. Assert "Sessions" heading inside the tabpanel.</t>
+  </si>
+  <si>
+    <t>Heading visible.</t>
+  </si>
+  <si>
+    <t>Original spec also asserted on "Current" session marker — relaxed because sessions list can be empty on a fresh login.</t>
+  </si>
+  <si>
+    <t>MA0005</t>
+  </si>
+  <si>
+    <t>Password section exposes Current/New inputs + Sign-out-other-sessions checkbox + Change password button</t>
+  </si>
+  <si>
+    <t>Security tab's password-change form renders all expected controls.</t>
+  </si>
+  <si>
+    <t>Security tab active.</t>
+  </si>
+  <si>
+    <t>1. Assert sessions heading, password heading, current pw, new pw, checkbox, change pw button.</t>
+  </si>
+  <si>
+    <t>All six controls visible.</t>
+  </si>
+  <si>
+    <t>MA0006</t>
+  </si>
+  <si>
+    <t>Clicking Change password with empty fields keeps the user on the page (no destructive call)</t>
+  </si>
+  <si>
+    <t>Surface check: form does not navigate or invalidate session on empty submit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Change password without typing anything.
+2. Assert URL still /manage-account.
+3. Assert current-password input still present.</t>
+  </si>
+  <si>
+    <t>No navigation; form persists.</t>
+  </si>
+  <si>
+    <t>We deliberately do not exercise a real password change — the test account is shared.</t>
+  </si>
+  <si>
+    <t>MA0007</t>
+  </si>
+  <si>
+    <t>Switching back to User details tab restores the name form</t>
+  </si>
+  <si>
+    <t>Tab navigation works bidirectionally.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click User details tab.
+2. Assert First/Last/Save visible.</t>
+  </si>
+  <si>
+    <t>User details form restored.</t>
+  </si>
+  <si>
+    <t>NV0001</t>
+  </si>
+  <si>
+    <t>Session persists across a full page reload</t>
+  </si>
+  <si>
+    <t>Refreshing the tickets dashboard must NOT log the user out.</t>
+  </si>
+  <si>
+    <t>Signed in on /&lt;slug&gt;/tickets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Reload page.
+2. Assert core chrome visible.
+3. Assert URL still in /&lt;slug&gt;/tickets.</t>
+  </si>
+  <si>
+    <t>Page rerenders signed-in.</t>
+  </si>
+  <si>
+    <t>Session</t>
+  </si>
+  <si>
+    <t>e2e/tests/navigation.spec.ts</t>
+  </si>
+  <si>
+    <t>NV0002</t>
+  </si>
+  <si>
+    <t>Navigating to /onboarding while signed in with an org redirects to /&lt;slug&gt;/tickets</t>
+  </si>
+  <si>
+    <t>Onboarding page is short-circuited when the user already belongs to an org.</t>
+  </si>
+  <si>
+    <t>User has an org.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to /onboarding.
+2. Wait for redirect.
+3. Assert URL matches /&lt;slug&gt;/tickets.</t>
+  </si>
+  <si>
+    <t>Redirect occurs.</t>
+  </si>
+  <si>
+    <t>NV0003</t>
+  </si>
+  <si>
+    <t>User-menu dropdown lists "Manage account" and "Sign out"</t>
+  </si>
+  <si>
+    <t>Header avatar dropdown shows the two expected options.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click avatar.
+2. Assert both menu items visible.
+3. Press Escape.</t>
+  </si>
+  <si>
+    <t>Menu shows both items.</t>
+  </si>
+  <si>
+    <t>NV0004</t>
+  </si>
+  <si>
+    <t>Sign out returns user to home, clears session, and blocks protected URLs</t>
+  </si>
+  <si>
+    <t>Full sign-out flow: UI click → redirect → cookie cleared → protected URL blocked.</t>
+  </si>
+  <si>
+    <t>Isolated browser context with a fresh sign-in.</t>
+  </si>
+  <si>
+    <t>Credentials.valid.{email,password}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. New isolated context.
+2. Sign in via UI.
+3. Click avatar &gt; Sign out.
+4. Assert URL is /.
+5. Assert anon header present.
+6. Try protected URL — assert NOT on it.</t>
+  </si>
+  <si>
+    <t>Session cleared; protected URLs blocked.</t>
+  </si>
+  <si>
+    <t>Runs in isolated context so it does not invalidate the shared storage-state cookie that other specs reuse.</t>
+  </si>
+  <si>
+    <t>NV0005</t>
+  </si>
+  <si>
+    <t>Org switcher dropdown shows current org and a "Create organization" option</t>
+  </si>
+  <si>
+    <t>Org switcher lists current org (disabled menu entry) and a create-new option.</t>
+  </si>
+  <si>
+    <t>Current org name.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click org switcher.
+2. Assert "Create organization" option.
+3. Assert current-org name appears.
+4. Press Escape.</t>
+  </si>
+  <si>
+    <t>Menu has both entries.</t>
+  </si>
+  <si>
     <t>AS0001</t>
   </si>
   <si>
@@ -466,6 +1294,132 @@
   </si>
   <si>
     <t>400 with details paths covering both required fields.</t>
+  </si>
+  <si>
+    <t>AT0001</t>
+  </si>
+  <si>
+    <t>Tickets API</t>
+  </si>
+  <si>
+    <t>Valid payload returns the new ticket with status "New"</t>
+  </si>
+  <si>
+    <t>Anonymous public ticket-submit endpoint creates a ticket scoped to the org named by x-organization.</t>
+  </si>
+  <si>
+    <t>Network reachable; org slug known.</t>
+  </si>
+  <si>
+    <t>qa-exploration-org slug + valid payload.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST tickets.create with valid payload + x-organization header.
+2. Assert 200.
+3. Assert body.status="New", title matches input, id matches /^[a-z0-9]+$/.</t>
+  </si>
+  <si>
+    <t>Ticket returned with status New.</t>
+  </si>
+  <si>
+    <t>api/tests/tickets.spec.ts</t>
+  </si>
+  <si>
+    <t>AT0002</t>
+  </si>
+  <si>
+    <t>Missing all required fields returns 400 with zod fieldErrors</t>
+  </si>
+  <si>
+    <t>Schema validation reports every missing field individually.</t>
+  </si>
+  <si>
+    <t>{} inner JSON.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST with empty inner json.
+2. Assert 400 BAD_REQUEST.
+3. Assert fieldErrors contains title, body, reportedBy, authorName.</t>
+  </si>
+  <si>
+    <t>All four field paths reported.</t>
+  </si>
+  <si>
+    <t>AT0003</t>
+  </si>
+  <si>
+    <t>Invalid email in reportedBy returns 400 with zod fieldErrors</t>
+  </si>
+  <si>
+    <t>Email validation surfaces as fieldErrors.reportedBy = ["Invalid email"].</t>
+  </si>
+  <si>
+    <t>reportedBy="notanemail" + other valid fields.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST.
+2. Assert 400.
+3. Assert fieldErrors.reportedBy contains "Invalid email".</t>
+  </si>
+  <si>
+    <t>Email error reported in fieldErrors.</t>
+  </si>
+  <si>
+    <t>AT0004</t>
+  </si>
+  <si>
+    <t>Empty inner JSON returns 400 with zod formErrors "Required"</t>
+  </si>
+  <si>
+    <t>Missing the tRPC inner payload entirely surfaces as formErrors (not fieldErrors).</t>
+  </si>
+  <si>
+    <t>{} outer JSON (no "0" key).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST with completely empty body.
+2. Assert 400.
+3. Assert formErrors=["Required"].</t>
+  </si>
+  <si>
+    <t>formErrors path set.</t>
+  </si>
+  <si>
+    <t>AT0005</t>
+  </si>
+  <si>
+    <t>Missing x-organization header returns 403 FORBIDDEN</t>
+  </si>
+  <si>
+    <t>The endpoint scopes to an org via the header; without it the request is forbidden.</t>
+  </si>
+  <si>
+    <t>Valid payload, NO x-organization header.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST without x-organization.
+2. Assert 403.
+3. Assert body.data.code="FORBIDDEN".</t>
+  </si>
+  <si>
+    <t>FORBIDDEN response.</t>
+  </si>
+  <si>
+    <t>AT0006</t>
+  </si>
+  <si>
+    <t>Unknown organization slug returns 403 FORBIDDEN</t>
+  </si>
+  <si>
+    <t>Unknown slug also returns FORBIDDEN (no enumeration leak).</t>
+  </si>
+  <si>
+    <t>x-organization="nonexistent-org-9921".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST with unknown slug.
+2. Assert 403.
+3. Assert body.data.code="FORBIDDEN".</t>
   </si>
 </sst>
 </file>
@@ -851,7 +1805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="16" customWidth="1"/>
@@ -1463,6 +2417,1956 @@
         <v>31</v>
       </c>
     </row>
+    <row r="13" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P27" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O28" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O29" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="P30" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O31" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="P31" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O32" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="P32" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O33" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P33" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O34" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P34" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O35" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P35" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O36" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P36" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O37" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P37" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P38" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="P39" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P41" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P42" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O43" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P43" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P44" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P45" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O46" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P46" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="M47" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O47" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="P47" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="P48" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="P49" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="P50" s="2" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="P51" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1471,7 +4375,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="16" customWidth="1"/>
@@ -1535,28 +4439,28 @@
     </row>
     <row r="2" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>351</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>100</v>
+        <v>353</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>101</v>
+        <v>354</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>102</v>
+        <v>355</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>103</v>
+        <v>356</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>104</v>
+        <v>357</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>105</v>
+        <v>358</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>86</v>
@@ -1577,7 +4481,7 @@
         <v>29</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>31</v>
@@ -1585,28 +4489,28 @@
     </row>
     <row r="3" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>107</v>
+        <v>360</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>108</v>
+        <v>361</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>109</v>
+        <v>362</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>90</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>111</v>
+        <v>364</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>112</v>
+        <v>365</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>24</v>
@@ -1627,7 +4531,7 @@
         <v>29</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>31</v>
@@ -1635,28 +4539,28 @@
     </row>
     <row r="4" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>113</v>
+        <v>366</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>114</v>
+        <v>367</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>115</v>
+        <v>368</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>96</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>111</v>
+        <v>364</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>116</v>
+        <v>369</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>39</v>
@@ -1677,7 +4581,7 @@
         <v>29</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>31</v>
@@ -1685,28 +4589,28 @@
     </row>
     <row r="5" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>117</v>
+        <v>370</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>118</v>
+        <v>371</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>119</v>
+        <v>372</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>120</v>
+        <v>373</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>121</v>
+        <v>374</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>122</v>
+        <v>375</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>39</v>
@@ -1727,7 +4631,7 @@
         <v>29</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>31</v>
@@ -1735,28 +4639,28 @@
     </row>
     <row r="6" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>123</v>
+        <v>376</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>124</v>
+        <v>377</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>125</v>
+        <v>378</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>126</v>
+        <v>379</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>127</v>
+        <v>380</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>128</v>
+        <v>381</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>39</v>
@@ -1777,7 +4681,7 @@
         <v>29</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>31</v>
@@ -1785,28 +4689,28 @@
     </row>
     <row r="7" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>129</v>
+        <v>382</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>130</v>
+        <v>383</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>131</v>
+        <v>384</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>132</v>
+        <v>385</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>133</v>
+        <v>386</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>134</v>
+        <v>387</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>39</v>
@@ -1827,7 +4731,7 @@
         <v>29</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P7" s="2" t="s">
         <v>31</v>
@@ -1835,28 +4739,28 @@
     </row>
     <row r="8" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>135</v>
+        <v>388</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>136</v>
+        <v>389</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>137</v>
+        <v>390</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>138</v>
+        <v>391</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>139</v>
+        <v>392</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>140</v>
+        <v>393</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>39</v>
@@ -1877,9 +4781,309 @@
         <v>29</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>106</v>
+        <v>359</v>
       </c>
       <c r="P8" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="P14" s="2" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>